<commit_message>
[tc-night] DSR-585/586 re-baseline ver0.4 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjT8AVkcXewLU2gDAqbae7
</commit_message>
<xml_diff>
--- a/ykk-dsr/hub/tc-out/[Sutrix] DSR -585- [AEM] 製品CF 改修（項目fix版対応）.xlsx
+++ b/ykk-dsr/hub/tc-out/[Sutrix] DSR -585- [AEM] 製品CF 改修（項目fix版対応）.xlsx
@@ -1423,7 +1423,7 @@
     <row r="11" ht="15.75" customHeight="1" s="48">
       <c r="A11" s="79" t="inlineStr">
         <is>
-          <t>製品CF 改修 / Product CF model (DM_product) – fixed field set (110→85), tags, import template; DSR-585 (related DSR-584/586/182/588), BL-OVL-1</t>
+          <t>製品CF 改修 / Product CF model (DM_product) – oracle DM_product_ver0.4 (83 fields, Quentin 20/10 comment 61605); DSR-585 (related DSR-584/586/182/588), BL-OVL-1</t>
         </is>
       </c>
       <c r="B11" s="79" t="n"/>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C12" s="95" t="inlineStr">
         <is>
-          <t>EN: Verify the product CF editor shows exactly the fields of the fixed list (85). JP: 製品CF編集画面に項目fix版の85項目が過不足なく表示されることを確認する。</t>
+          <t>EN: Verify the product CF editor shows exactly the 83 fields of DM_product_ver0.4 (sheet 製品CF（0.4）). JP: 製品CF編集画面にDM_product_ver0.4の83項目が過不足なく表示されることを確認する。</t>
         </is>
       </c>
       <c r="D12" s="95" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="E12" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. Open TD-585-01 in the CF editor. 2. Expand all tabs. 3. List every field label + name. 4. Compare with the fixed field list (oracle: 項目fix版; provisional 20260930_製品CFフィールド再整理_v0.1.xlsx – A1). JP: 1. 開く 2. 全タブ展開 3. 項目一覧 4. fix版と比較。</t>
+          <t>EN: 1. Open TD-585-01 in the CF editor. 2. Expand all 10 tabs (基本情報, 検索・分類, 表示情報, Media01, Media02, Media03, 詳細, 製品情報, 関連情報, 管理情報). 3. List every field label + name. 4. Compare with sheet 製品CF（0.4） rows 1-1 … 10-4 (oracle A1). JP: 1. 開く 2. 10タブ展開 3. 項目一覧 4. ver0.4と比較。</t>
         </is>
       </c>
       <c r="F12" s="95" t="inlineStr">
         <is>
-          <t>EN: Field count = 85 (or the count in the fix list); every fix-list name present; no extra field. Differences listed. JP: 85項目、過不足なし。</t>
+          <t>EN: 10 tabs in this order; 83 fields (basic 3, search 5, display 5, Media01 14, Media02 15, Media03 15, detail 11, product info 6, related 5, management 4); every ver0.4 name present, 0 extra; no 生産情報 tab. Differences listed. JP: 10タブ・83項目、過不足なし、生産情報タブなし。</t>
         </is>
       </c>
       <c r="G12" s="95" t="n"/>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="U12" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V12" s="59" t="n"/>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="C13" s="95" t="inlineStr">
         <is>
-          <t>EN: Verify fields removed in the fix list are not shown in the editor. JP: 削除項目が編集画面に表示されないことを確認する。</t>
+          <t>EN: Verify the 27 fields removed in ver0.3→0.4 (差分管理 2026-10-06) are not in the editor. JP: ver0.3→0.4で削除された27項目が編集画面にないことを確認する。</t>
         </is>
       </c>
       <c r="D13" s="95" t="inlineStr">
@@ -1571,12 +1571,12 @@
       </c>
       <c r="E13" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. In TD-585-01 search the editor for each removed field (v0.1 構築断念 examples: itemManager, materials, appearances, sewingSuitabilities, salesOffices, moq, orderLot, careDry, careWash, productionCountries, leadTime). JP: 削除項目を検索。</t>
+          <t>EN: 1. In TD-585-01 search the editor (all tabs) for each removed name: itemManager, materials, appearances, sewingSuitabilities, plasticHardwareFunctionCategories, salesOffices, isStandardItem, certifications, internalCertifications, reverseUse, reversible, topBottomStopVariation, moq, orderLot, qualityStandards, qualityStandardDescription, careDry, careWash, careIron, sustainabilityText, productionCountries, productionCompany, dailyProductionCapacity, leadTime, developmentCompany, applicableSliderStandard, applicableSliderSpecial. 2. Also check the old spellings Notice, NoticeImage, Howtouse, HowtouseImage. JP: 削除27項目と旧表記を検索。</t>
         </is>
       </c>
       <c r="F13" s="95" t="inlineStr">
         <is>
-          <t>EN: None of the removed fields is visible in any tab. JP: いずれも表示されない。</t>
+          <t>EN: 0 of the 27 removed fields and 0 old spellings visible in any tab (renamed fields appear as notice / noticeImage / howToUse / howToUseImage). JP: いずれも表示されない。</t>
         </is>
       </c>
       <c r="G13" s="95" t="n"/>
@@ -1598,7 +1598,7 @@
       <c r="K13" s="95" t="n"/>
       <c r="L13" s="96" t="inlineStr">
         <is>
-          <t>BAC#1; TCC#1</t>
+          <t>差分管理 0.3→0.4 (削除); TCC#1</t>
         </is>
       </c>
       <c r="M13" s="96" t="n"/>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="U13" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V13" s="59" t="n"/>
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E14" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. For each field, record editor widget: text / multiline / tag picker / boolean / date / number / enumeration / asset ref. 2. Compare with fix-list type column. JP: 型を記録し比較。</t>
+          <t>EN: 1. For each field record the editor widget. 2. Compare with the type column of 製品CF（0.4）. JP: 型を記録しver0.4と比較。</t>
         </is>
       </c>
       <c r="F14" s="95" t="inlineStr">
         <is>
-          <t>EN: Text(255) = single-line; 長文 = multiline; タグ = tag picker (multi); ○ = boolean; YYYY-MM-DD = date; 数値 = number; 選択 = enumeration; DAM path = content/asset reference. 0 mismatch. JP: 型不一致0件。</t>
+          <t>EN: single line text → single-line; multi line text (Plain) → plain multiline (description, colorVariations, howToUse, notice); multi line text (Rich Text) → RTE (itemVariations); Tag / Tag（複数） → tag picker (productCategories single; applications, performances, zipperChainTypeCategories multi); boolean → checkbox/switch with default False (isDtmSupported, is3dSimulatorSupported, printableTape, recycledTape, recycledMaterial, isDiscontinued); asset reference → asset picker; URL → URL field (mediaNNUrl); fragment reference（複数）→ multi CF picker (parentProduct, relatedProducts, relatedCatalogs, relatedVideos); number → sortOrder default 0; Date and Time (Date Only) → publishDate, updateDate. openingType: see 7.0. 0 mismatch. JP: 型不一致0件。</t>
         </is>
       </c>
       <c r="G14" s="95" t="n"/>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="U14" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V14" s="59" t="n"/>
@@ -1759,12 +1759,12 @@
       </c>
       <c r="E15" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. Clear one required field (productId, productCode, productName, productCategories, applications, media01Asset, publishDate – fix list ※). 2. Save. 3. Restore and repeat for the next field. JP: 必須を1つずつ空にして保存。</t>
+          <t>EN: 1. Clear one required field of ver0.4 (必須 ○): productId, productCode, productName, productCategories, applications, media01Asset, publishDate. 2. Save. 3. Restore and repeat for the next field. 4. Leave one optional field empty (e.g. performances) and save. JP: 必須7項目を1つずつ空にして保存、任意項目は空で保存。</t>
         </is>
       </c>
       <c r="F15" s="95" t="inlineStr">
         <is>
-          <t>EN: Each time a required-field error is shown and save/publish is blocked; optional fields left empty do not block. JP: 毎回エラー、任意項目は保存可。</t>
+          <t>EN: For each of the 7 required fields a required-field error is shown and save/publish is blocked; the optional field left empty saves OK. JP: 必須7項目は毎回エラー、任意項目は保存可。</t>
         </is>
       </c>
       <c r="G15" s="95" t="n"/>
@@ -1786,7 +1786,7 @@
       <c r="K15" s="95" t="n"/>
       <c r="L15" s="96" t="inlineStr">
         <is>
-          <t>TCC#1 (required flags)</t>
+          <t>ver0.4 必須 column; TCC#1</t>
         </is>
       </c>
       <c r="M15" s="96" t="n"/>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="U15" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V15" s="59" t="n"/>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="F16" s="95" t="inlineStr">
         <is>
-          <t>EN: 255 saved unchanged; 256 → error or input stops at 255 (record which). JP: 255字保存、256字はエラーまたは入力制限。</t>
+          <t>EN: 255 chars saved unchanged. 256 chars: record behaviour (error / truncation / saved) – ver0.4 defines no max length (A6), so Fail only if 255 chars are rejected or changed. JP: 255字は保存。256字は挙動を記録（ver0.4に上限定義なし）。</t>
         </is>
       </c>
       <c r="G16" s="95" t="n"/>
@@ -1880,7 +1880,7 @@
       <c r="K16" s="95" t="n"/>
       <c r="L16" s="96" t="inlineStr">
         <is>
-          <t>Fix list type テキスト（最大255字）</t>
+          <t>ver0.4 single line text; A6 boundary</t>
         </is>
       </c>
       <c r="M16" s="96" t="n"/>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="U16" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V16" s="59" t="n"/>
@@ -1947,12 +1947,12 @@
       </c>
       <c r="E17" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. In TD-585-01 open the zipperChainTypeCategories picker. 2. Select 2 tags (e.g. CN, and one more). 3. Save, reopen. JP: 2つ選択し保存、再表示。</t>
+          <t>EN: 1. In TD-585-01 open the zipperChainTypeCategories picker. 2. Record the tag names shown. 3. Select 2 tags. 4. Save, reopen. JP: タグ名を記録、2つ選択し保存、再表示。</t>
         </is>
       </c>
       <c r="F17" s="95" t="inlineStr">
         <is>
-          <t>EN: Picker lists only chain-type tags; both tags kept after reopen. JP: チェーンタイプのタグのみ、2つ保持。</t>
+          <t>EN: Picker lists only chain-type tags; tag names follow the 10/6 rule = size digits + 2-letter chain type (e.g. 5CN) – names that do not follow it are listed; both selected tags kept after reopen. JP: チェーンタイプのタグのみ（数字＋英字2文字）、2つ保持。</t>
         </is>
       </c>
       <c r="G17" s="95" t="n"/>
@@ -1974,7 +1974,7 @@
       <c r="K17" s="95" t="n"/>
       <c r="L17" s="96" t="inlineStr">
         <is>
-          <t>DSR-585 scope (タグ項目); TCC#1</t>
+          <t>ver0.4 2-4 + 差分管理 10/6 (タグは2文字の系統)</t>
         </is>
       </c>
       <c r="M17" s="96" t="n"/>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="U17" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin + tag namespace</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V17" s="59" t="n"/>
@@ -2026,12 +2026,12 @@
       </c>
       <c r="B18" s="95" t="inlineStr">
         <is>
-          <t>Enumeration – openingType values</t>
+          <t>openingType – values (Enumeration multiple)</t>
         </is>
       </c>
       <c r="C18" s="95" t="inlineStr">
         <is>
-          <t>EN: Verify openingType offers only the defined values. JP: ファスナー製品仕様の選択肢が定義どおりであることを確認する。</t>
+          <t>EN: Verify openingType offers the 4 defined values and stores several. JP: ファスナー製品仕様が4値の複数選択であることを確認する。</t>
         </is>
       </c>
       <c r="D18" s="95" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="E18" s="95" t="inlineStr">
         <is>
-          <t>EN: 1. Open the openingType dropdown. 2. Record options. JP: 選択肢を記録。</t>
+          <t>EN: 1. Open openingType in TD-585-01. 2. Record widget type and options. 3. Select 止 and 開, save, reopen. JP: 型・選択肢を記録、2つ選択し保存。</t>
         </is>
       </c>
       <c r="F18" s="95" t="inlineStr">
         <is>
-          <t>EN: Options = fix list values (v0.1: stop / open / reverseOpen / chain), no others. JP: fix版の値のみ。</t>
+          <t>EN: Multi-select enumeration with exactly 止 / 開 / 逆開 / チェーン (or their stored values stop/open/reverseOpen/chain); both selections kept. If the field is single line text (open customer request, A7/Q45) → record as Pending, not Fail. JP: 4値・複数選択。single line textならPending。</t>
         </is>
       </c>
       <c r="G18" s="95" t="n"/>
@@ -2068,7 +2068,7 @@
       <c r="K18" s="95" t="n"/>
       <c r="L18" s="96" t="inlineStr">
         <is>
-          <t>Fix list (選択)</t>
+          <t>ver0.4 3-4; 差分管理 0.3→0.4</t>
         </is>
       </c>
       <c r="M18" s="96" t="n"/>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="U18" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V18" s="59" t="n"/>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="F19" s="95" t="inlineStr">
         <is>
-          <t>EN: Same set of names (0 missing, 0 extra); required columns marked ※; version/date in file name newer than v1.1_20260914. JP: 列一致、必須表示、版更新。</t>
+          <t>EN: Same set of names as ver0.4 (83, 0 missing, 0 extra); required columns marked ※/○ (7); version/date in file name newer than v1.1_20260914. JP: 列一致、必須7列表示、版更新。</t>
         </is>
       </c>
       <c r="G19" s="95" t="n"/>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="U19" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin + template revision (Chiba)</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat · template revision + import procedure (Q28, Chiba)</t>
         </is>
       </c>
       <c r="V19" s="59" t="n"/>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="U20" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin · import procedure (Q28)</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat · template revision + import procedure (Q28, Chiba)</t>
         </is>
       </c>
       <c r="V20" s="59" t="n"/>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="U21" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin · import procedure (Q28)</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat · template revision + import procedure (Q28, Chiba)</t>
         </is>
       </c>
       <c r="V21" s="59" t="n"/>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="U22" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V22" s="59" t="n"/>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="U23" s="97" t="inlineStr">
         <is>
-          <t>cn folder may not exist (Issue #18) · 項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin</t>
+          <t>cn folder may not exist (Issue #18) · DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V23" s="59" t="n"/>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="F24" s="95" t="inlineStr">
         <is>
-          <t>EN: HTTP 200; productName, zipperChainTypeCategories, publishDate present with TD values; none of the removed field names present. JP: 新項目あり、削除項目なし。</t>
+          <t>EN: HTTP 200, no 'errors'; product contains productId, productCode, productName, publishDate with TD values and the ver0.4 detail fields (itemVariationsImage, colorVariationsImage, howToUse, howToUseImage, recycledMaterial, recycledMaterialNote, applicableSliderSameAsParent, parentProduct, notice, noticeImage); none of the 27 removed names and none of Howtouse / HowtouseImage / Notice / NoticeImage. JP: ver0.4項目あり、削除項目・旧表記なし。</t>
         </is>
       </c>
       <c r="G24" s="95" t="n"/>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="U24" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin · query update DSR-586 (Martin)</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
         </is>
       </c>
       <c r="V24" s="59" t="n"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="F25" s="95" t="inlineStr">
         <is>
-          <t>EN: Entry found; keys include productId/productName/productCategories/applications; no removed field keys. JP: 必要キーあり、削除項目なし。</t>
+          <t>EN: Entry found; keys include productId/productName/productCategories/applications; none of the 27 removed field names (A1). JP: 必要キーあり、削除項目なし。</t>
         </is>
       </c>
       <c r="G25" s="95" t="n"/>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="U25" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin · DSR-560/182 (Nakamoto)</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat · DSR-560/182 (Nakamoto)</t>
         </is>
       </c>
       <c r="V25" s="59" t="n"/>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="U26" s="97" t="inlineStr">
         <is>
-          <t>項目fix版 from YKK (due 10/14, not delivered 10/16) + DM_product model update (Chiba) – owner Quentin · DSR-586 [Dev] In Testing (Martin)</t>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat · DSR-586 overlay (Martin)</t>
         </is>
       </c>
       <c r="V26" s="59" t="n"/>
@@ -2865,39 +2865,91 @@
       <c r="AB26" s="59" t="n"/>
     </row>
     <row r="27" ht="187.5" customHeight="1" s="48">
-      <c r="A27" s="84" t="n"/>
-      <c r="B27" s="84" t="n"/>
-      <c r="C27" s="84" t="n"/>
-      <c r="D27" s="84" t="n"/>
-      <c r="E27" s="84" t="n"/>
-      <c r="F27" s="84" t="n"/>
-      <c r="G27" s="84" t="n"/>
-      <c r="H27" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="I27" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="J27" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="K27" s="84" t="n"/>
-      <c r="L27" s="58" t="n"/>
-      <c r="M27" s="57" t="n"/>
-      <c r="N27" s="57" t="n"/>
-      <c r="O27" s="57" t="n"/>
-      <c r="P27" s="87" t="n"/>
-      <c r="Q27" s="87" t="n"/>
-      <c r="R27" s="87" t="n"/>
-      <c r="S27" s="87" t="n"/>
-      <c r="T27" s="87" t="n"/>
-      <c r="U27" s="87" t="n"/>
+      <c r="A27" s="95" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="B27" s="95" t="inlineStr">
+        <is>
+          <t>Media slots – media01 image fixed, media02–15 Type/Asset/Url</t>
+        </is>
+      </c>
+      <c r="C27" s="95" t="inlineStr">
+        <is>
+          <t>EN: Verify media01 is an image-only asset field and media02–15 each have Type (Image/Video/360/3D/External), Asset and Url. JP: media01は画像固定、media02〜15は種別・アセット・URLを持つことを確認する。</t>
+        </is>
+      </c>
+      <c r="D27" s="95" t="inlineStr">
+        <is>
+          <t>EN: DM_product ver0.4 on DEV Author; TD-585-01 exists. JP: ver0.4反映済み、TD-585-01。</t>
+        </is>
+      </c>
+      <c r="E27" s="95" t="inlineStr">
+        <is>
+          <t>EN: 1. Media01 tab: check photoForList and media01Asset (no Type field). 2. In media01Asset try to pick a video asset. 3. For media02…media15 record the 3 fields and the Type options. 4. Set media02Type=External + media02Url=https://www.ykkfastening.com/ , save, reopen. JP: 各スロットの項目と選択肢を記録、External+URLを保存。</t>
+        </is>
+      </c>
+      <c r="F27" s="95" t="inlineStr">
+        <is>
+          <t>EN: media01 has no Type field; media01Asset accepts images (video rejected or not listed – record); each of media02–15 has Type with exactly Image/Video/360/3D/External, Asset and Url; External + URL saved and kept. JP: media01は画像のみ、02〜15は3項目・5種別、保存保持。</t>
+        </is>
+      </c>
+      <c r="G27" s="95" t="n"/>
+      <c r="H27" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="I27" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="J27" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="K27" s="95" t="n"/>
+      <c r="L27" s="96" t="inlineStr">
+        <is>
+          <t>ver0.4 4-1…6-15; BL note 20/10 15:20</t>
+        </is>
+      </c>
+      <c r="M27" s="96" t="n"/>
+      <c r="N27" s="97" t="n"/>
+      <c r="O27" s="97" t="n"/>
+      <c r="P27" s="97" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="Q27" s="97" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="R27" s="97" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="S27" s="97" t="inlineStr">
+        <is>
+          <t>AEM Author (Chrome)</t>
+        </is>
+      </c>
+      <c r="T27" s="97" t="inlineStr">
+        <is>
+          <t>TD-585-01</t>
+        </is>
+      </c>
+      <c r="U27" s="97" t="inlineStr">
+        <is>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
+        </is>
+      </c>
       <c r="V27" s="59" t="n"/>
       <c r="W27" s="59" t="n"/>
       <c r="X27" s="59" t="n"/>
@@ -2907,39 +2959,91 @@
       <c r="AB27" s="59" t="n"/>
     </row>
     <row r="28" ht="187.5" customHeight="1" s="48">
-      <c r="A28" s="84" t="n"/>
-      <c r="B28" s="84" t="n"/>
-      <c r="C28" s="84" t="n"/>
-      <c r="D28" s="84" t="n"/>
-      <c r="E28" s="84" t="n"/>
-      <c r="F28" s="84" t="n"/>
-      <c r="G28" s="84" t="n"/>
-      <c r="H28" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="I28" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="J28" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="K28" s="84" t="n"/>
-      <c r="L28" s="85" t="n"/>
-      <c r="M28" s="86" t="n"/>
-      <c r="N28" s="57" t="n"/>
-      <c r="O28" s="57" t="n"/>
-      <c r="P28" s="87" t="n"/>
-      <c r="Q28" s="87" t="n"/>
-      <c r="R28" s="87" t="n"/>
-      <c r="S28" s="87" t="n"/>
-      <c r="T28" s="87" t="n"/>
-      <c r="U28" s="87" t="n"/>
+      <c r="A28" s="95" t="inlineStr">
+        <is>
+          <t>17.0</t>
+        </is>
+      </c>
+      <c r="B28" s="95" t="inlineStr">
+        <is>
+          <t>New ver0.4 fields – types and defaults</t>
+        </is>
+      </c>
+      <c r="C28" s="95" t="inlineStr">
+        <is>
+          <t>EN: Verify the 7 fields added in ver0.3→0.4 exist with the defined type and default. JP: ver0.4追加7項目が定義どおりの型・初期値であることを確認する。</t>
+        </is>
+      </c>
+      <c r="D28" s="95" t="inlineStr">
+        <is>
+          <t>EN: DM_product ver0.4 on DEV Author; TD-585-01 exists. JP: ver0.4反映済み、TD-585-01。</t>
+        </is>
+      </c>
+      <c r="E28" s="95" t="inlineStr">
+        <is>
+          <t>EN: 1. In a NEW CF TD-585-02 (before filling) record type and default of: itemVariationsImage, colorVariationsImage, howToUse, howToUseImage, recycledMaterial, recycledMaterialNote, applicableSliderSameAsParent. 2. Fill each (images: any QA image; recycledMaterial ON; texts 'QA585 …'). 3. Save, reopen. JP: 型・初期値を記録、入力して保存・再表示。</t>
+        </is>
+      </c>
+      <c r="F28" s="95" t="inlineStr">
+        <is>
+          <t>EN: itemVariationsImage, colorVariationsImage, howToUseImage = asset reference; howToUse = plain multiline; recycledMaterial = boolean default False; recycledMaterialNote = single-line; applicableSliderSameAsParent = single enumeration with option 'any' and empty allowed; all values kept after reopen. JP: 型・初期値一致、値保持。</t>
+        </is>
+      </c>
+      <c r="G28" s="95" t="n"/>
+      <c r="H28" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="I28" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="J28" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="K28" s="95" t="n"/>
+      <c r="L28" s="96" t="inlineStr">
+        <is>
+          <t>差分管理 0.3→0.4 (追加); ver0.4 7-4, 7-6, 7-8, 7-9, 8-5, 8-6, 9-2</t>
+        </is>
+      </c>
+      <c r="M28" s="96" t="n"/>
+      <c r="N28" s="97" t="n"/>
+      <c r="O28" s="97" t="n"/>
+      <c r="P28" s="97" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="Q28" s="97" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="R28" s="97" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="S28" s="97" t="inlineStr">
+        <is>
+          <t>AEM Author (Chrome)</t>
+        </is>
+      </c>
+      <c r="T28" s="97" t="inlineStr">
+        <is>
+          <t>TD-585-02</t>
+        </is>
+      </c>
+      <c r="U28" s="97" t="inlineStr">
+        <is>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
+        </is>
+      </c>
       <c r="V28" s="59" t="n"/>
       <c r="W28" s="59" t="n"/>
       <c r="X28" s="59" t="n"/>
@@ -2949,39 +3053,91 @@
       <c r="AB28" s="59" t="n"/>
     </row>
     <row r="29" ht="187.5" customHeight="1" s="48">
-      <c r="A29" s="84" t="n"/>
-      <c r="B29" s="84" t="n"/>
-      <c r="C29" s="84" t="n"/>
-      <c r="D29" s="84" t="n"/>
-      <c r="E29" s="84" t="n"/>
-      <c r="F29" s="84" t="n"/>
-      <c r="G29" s="84" t="n"/>
-      <c r="H29" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="I29" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="J29" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="K29" s="84" t="n"/>
-      <c r="L29" s="85" t="n"/>
-      <c r="M29" s="86" t="n"/>
-      <c r="N29" s="57" t="n"/>
-      <c r="O29" s="57" t="n"/>
-      <c r="P29" s="87" t="n"/>
-      <c r="Q29" s="87" t="n"/>
-      <c r="R29" s="87" t="n"/>
-      <c r="S29" s="87" t="n"/>
-      <c r="T29" s="87" t="n"/>
-      <c r="U29" s="87" t="n"/>
+      <c r="A29" s="95" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
+      <c r="B29" s="95" t="inlineStr">
+        <is>
+          <t>CF name = productId digits, content CF folder</t>
+        </is>
+      </c>
+      <c r="C29" s="95" t="inlineStr">
+        <is>
+          <t>EN: Verify product content CFs are stored in /content/dam/common/{lang}/products/ with name = productId (digits, no prefix). JP: 製品CFが/content/dam/common/{lang}/products/にproductIdと同じ番号名で保存されることを確認する。</t>
+        </is>
+      </c>
+      <c r="D29" s="95" t="inlineStr">
+        <is>
+          <t>EN: DM_product ver0.4 on DEV Author; TD-585-01 exists. JP: ver0.4反映済み、TD-585-01。</t>
+        </is>
+      </c>
+      <c r="E29" s="95" t="inlineStr">
+        <is>
+          <t>EN: 1. Open TD-585-01: record CF path, name and productId value. 2. List the folder /content/dam/common/ja/products and record up to 10 names. JP: パス・名前・productIdを記録、フォルダ内の名前を記録。</t>
+        </is>
+      </c>
+      <c r="F29" s="95" t="inlineStr">
+        <is>
+          <t>EN: TD-585-01 path = /content/dam/common/ja/products/990585001 and productId = 990585001; names in the folder are digits only (others, e.g. productId-01x, listed as data to clean, not Fail of the model). JP: 名前=productId、数字のみ（例外は一覧化）。</t>
+        </is>
+      </c>
+      <c r="G29" s="95" t="n"/>
+      <c r="H29" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="I29" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="J29" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="K29" s="95" t="n"/>
+      <c r="L29" s="96" t="inlineStr">
+        <is>
+          <t>ver0.4 a2, 1-1; 差分管理 10/6</t>
+        </is>
+      </c>
+      <c r="M29" s="96" t="n"/>
+      <c r="N29" s="97" t="n"/>
+      <c r="O29" s="97" t="n"/>
+      <c r="P29" s="97" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="Q29" s="97" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="R29" s="97" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="S29" s="97" t="inlineStr">
+        <is>
+          <t>AEM Author (Chrome)</t>
+        </is>
+      </c>
+      <c r="T29" s="97" t="inlineStr">
+        <is>
+          <t>TD-585-01</t>
+        </is>
+      </c>
+      <c r="U29" s="97" t="inlineStr">
+        <is>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) + TD-585 seed (QA-PT) – owner Martin/Dat</t>
+        </is>
+      </c>
       <c r="V29" s="59" t="n"/>
       <c r="W29" s="59" t="n"/>
       <c r="X29" s="59" t="n"/>
@@ -2991,39 +3147,91 @@
       <c r="AB29" s="59" t="n"/>
     </row>
     <row r="30" ht="187.5" customHeight="1" s="48">
-      <c r="A30" s="84" t="n"/>
-      <c r="B30" s="84" t="n"/>
-      <c r="C30" s="84" t="n"/>
-      <c r="D30" s="84" t="n"/>
-      <c r="E30" s="84" t="n"/>
-      <c r="F30" s="84" t="n"/>
-      <c r="G30" s="84" t="n"/>
-      <c r="H30" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="I30" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="J30" s="84" t="inlineStr">
-        <is>
-          <t>To do / 未実施</t>
-        </is>
-      </c>
-      <c r="K30" s="84" t="n"/>
-      <c r="L30" s="85" t="n"/>
-      <c r="M30" s="86" t="n"/>
-      <c r="N30" s="57" t="n"/>
-      <c r="O30" s="57" t="n"/>
-      <c r="P30" s="87" t="n"/>
-      <c r="Q30" s="87" t="n"/>
-      <c r="R30" s="87" t="n"/>
-      <c r="S30" s="87" t="n"/>
-      <c r="T30" s="87" t="n"/>
-      <c r="U30" s="87" t="n"/>
+      <c r="A30" s="95" t="inlineStr">
+        <is>
+          <t>19.0</t>
+        </is>
+      </c>
+      <c r="B30" s="95" t="inlineStr">
+        <is>
+          <t>All product persisted queries use ver0.4 names</t>
+        </is>
+      </c>
+      <c r="C30" s="95" t="inlineStr">
+        <is>
+          <t>EN: Verify every product persisted query returns ver0.4 field names only. JP: 製品系persisted queryがver0.4の項目名のみ返すことを確認する。</t>
+        </is>
+      </c>
+      <c r="D30" s="95" t="inlineStr">
+        <is>
+          <t>EN: DM_product ver0.4 on DEV Author; TD-585-01 exists. JP: ver0.4反映済み、TD-585-01。</t>
+        </is>
+      </c>
+      <c r="E30" s="95" t="inlineStr">
+        <is>
+          <t>EN: 1. GET (publish, unencoded ;) dsr-product-page;path=/content/dam/dsr/ja/products/46, product-detail;productId=productId-01x, dsr-product-list;folder=/content/dam/dsr/ja/products/, dm-product-list. 2. Collect all field names of product items. JP: 4クエリを取得し項目名を収集。</t>
+        </is>
+      </c>
+      <c r="F30" s="95" t="inlineStr">
+        <is>
+          <t>EN: All 200 without 'errors'; 0 removed names (27); 0 old spellings (Howtouse, HowtouseImage, Notice, NoticeImage, applicableSliderStandard, applicableSliderSpecial). JOB-20261020-09 saw old names in product-detail → Fail if still present after Martin's done ping (Q46). JP: 削除項目・旧表記0件。</t>
+        </is>
+      </c>
+      <c r="G30" s="95" t="n"/>
+      <c r="H30" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="I30" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="J30" s="95" t="inlineStr">
+        <is>
+          <t>To do / 未実施</t>
+        </is>
+      </c>
+      <c r="K30" s="95" t="n"/>
+      <c r="L30" s="96" t="inlineStr">
+        <is>
+          <t>Incident 20/10; ver0.4; BL-OVL-1</t>
+        </is>
+      </c>
+      <c r="M30" s="96" t="n"/>
+      <c r="N30" s="97" t="n"/>
+      <c r="O30" s="97" t="n"/>
+      <c r="P30" s="97" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="Q30" s="97" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="R30" s="97" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="S30" s="97" t="inlineStr">
+        <is>
+          <t>API (Playwright request)</t>
+        </is>
+      </c>
+      <c r="T30" s="97" t="inlineStr">
+        <is>
+          <t>— (existing DEV data, read-only)</t>
+        </is>
+      </c>
+      <c r="U30" s="97" t="inlineStr">
+        <is>
+          <t>DM_product ver0.4 finished on DEV (Martin done ping – 🔔 P1 Dat) – owner Martin</t>
+        </is>
+      </c>
       <c r="V30" s="59" t="n"/>
       <c r="W30" s="59" t="n"/>
       <c r="X30" s="59" t="n"/>
@@ -5510,12 +5718,12 @@
       </c>
       <c r="B2" s="98" t="inlineStr">
         <is>
-          <t>項目fix版 (85 fields) not delivered as of 2026-10-16 (DSR-585 comments 60822, 61098). Provisional oracle = 20260930_製品CFフィールド再整理_v0.1.xlsx: 構築断念 = removed, MT改修待ち = changed, ※ = required. Replace with fix list when delivered; TC text stays.</t>
+          <t>Oracle = DM_product_ver0.4.xlsx sheet 製品CF（0.4） + 差分管理 (Drive 1uUgIMKKSL93jjVCQpfTTYtkrFJlAAiSD), confirmed by Quentin 2026-10-20 (DSR-585 comment 61605: earlier attached file was old). Replaces v0.1 and 項目fix版 1Rxiw3S… . 83 fields in 10 tabs; 7 required.</t>
         </is>
       </c>
       <c r="C2" s="98" t="inlineStr">
         <is>
-          <t>DSR-585; Drive v0.1</t>
+          <t>DSR-585 61605; ver0.4</t>
         </is>
       </c>
       <c r="D2" s="98" t="inlineStr">
@@ -5613,22 +5821,70 @@
       </c>
     </row>
     <row r="7" ht="29.25" customHeight="1" s="48">
-      <c r="A7" s="94" t="n"/>
-      <c r="B7" s="94" t="n"/>
-      <c r="C7" s="94" t="n"/>
-      <c r="D7" s="94" t="n"/>
+      <c r="A7" s="98" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B7" s="98" t="inlineStr">
+        <is>
+          <t>[Giả định] ver0.4 defines no max length for single line text; 5.0 only fails if 255 chars are rejected.</t>
+        </is>
+      </c>
+      <c r="C7" s="98" t="inlineStr">
+        <is>
+          <t>ver0.4</t>
+        </is>
+      </c>
+      <c r="D7" s="98" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="29.25" customHeight="1" s="48">
-      <c r="A8" s="94" t="n"/>
-      <c r="B8" s="94" t="n"/>
-      <c r="C8" s="94" t="n"/>
-      <c r="D8" s="94" t="n"/>
+      <c r="A8" s="98" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B8" s="98" t="inlineStr">
+        <is>
+          <t>[Giả định] openingType stays Enumeration（複数） (ver0.4); customer asked to change it to single line text (comment in ver0.4 3-4, Q45). If changed on DEV → 7.0 Pending and TC updated.</t>
+        </is>
+      </c>
+      <c r="C8" s="98" t="inlineStr">
+        <is>
+          <t>ver0.4 3-4</t>
+        </is>
+      </c>
+      <c r="D8" s="98" t="inlineStr">
+        <is>
+          <t>7.0, 3.0</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="48">
-      <c r="A9" s="94" t="n"/>
-      <c r="B9" s="94" t="n"/>
-      <c r="C9" s="94" t="n"/>
-      <c r="D9" s="94" t="n"/>
+      <c r="A9" s="98" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B9" s="98" t="inlineStr">
+        <is>
+          <t>Model on DEV changed twice on 2026-10-20 (DSR-585 CR 11:48–13:50 JST; ver0.4 by Martin from 17:14 JST). Results before Martin's done ping are not verdicts. New fields are parsed but not rendered (no design) → Page checks of new fields Blocked (see DSR-586 20.0).</t>
+        </is>
+      </c>
+      <c r="C9" s="98" t="inlineStr">
+        <is>
+          <t>Incident 20/10; BL-OVL-1 update 20/10</t>
+        </is>
+      </c>
+      <c r="D9" s="98" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>